<commit_message>
feat: EDA complete, DecisionTreeClassifier complete
</commit_message>
<xml_diff>
--- a/Data/Diccionario_Datos.xlsx
+++ b/Data/Diccionario_Datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\dell\Documents\Uniandes\MaIA\Principios del ML\Proyecto\2025-20\Etapa 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files 1\DOCUMENTOS JHON\CEREBRO DIGITAL\Maestría en IA Andes\Principios de Machine Learning\Modulo 7\Proyecto Etapa-2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEEEEF25-E3C4-44D6-9A9C-9B4CA3533A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B9D7BA-5B8C-4C80-9369-6513C38B1584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>Edad</t>
   </si>
@@ -113,6 +113,36 @@
   </si>
   <si>
     <t>Padecimiento de hipertensión (Sí, No)</t>
+  </si>
+  <si>
+    <t>Tipo variable</t>
+  </si>
+  <si>
+    <t>númerica</t>
+  </si>
+  <si>
+    <t>Numerica</t>
+  </si>
+  <si>
+    <t>Numérica</t>
+  </si>
+  <si>
+    <t>Categorica Ordinal</t>
+  </si>
+  <si>
+    <t>Categórica Nominal</t>
+  </si>
+  <si>
+    <t>Categórica Binaria</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Target</t>
   </si>
 </sst>
 </file>
@@ -145,15 +175,45 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFAB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -161,24 +221,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFFAB"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -507,140 +620,207 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.42578125" customWidth="1"/>
     <col min="2" max="2" width="78.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A2" s="1" t="s">
+      <c r="C2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="15" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A5" s="1" t="s">
+      <c r="C5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A6" s="1" t="s">
+      <c r="C6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="17"/>
+    </row>
+    <row r="7" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A7" s="1" t="s">
+      <c r="C7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A8" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="15" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A8" s="1" t="s">
+      <c r="C8" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="17"/>
+    </row>
+    <row r="9" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A9" s="1" t="s">
+      <c r="C9" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="10" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A10" s="1" t="s">
+      <c r="C10" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A11" s="1" t="s">
+      <c r="C11" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A12" s="1" t="s">
+      <c r="C12" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="24.95" customHeight="1">
+      <c r="A13" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="24.95" customHeight="1">
-      <c r="A13" s="1" t="s">
+      <c r="C13" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="B14" s="2"/>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="B16" s="2"/>
+      <c r="C14" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="B16" s="1"/>
     </row>
     <row r="18" spans="2:2">
-      <c r="B18" s="2"/>
+      <c r="B18" s="1"/>
     </row>
     <row r="20" spans="2:2">
-      <c r="B20" s="2"/>
+      <c r="B20" s="1"/>
     </row>
     <row r="22" spans="2:2">
-      <c r="B22" s="2"/>
+      <c r="B22" s="1"/>
     </row>
     <row r="24" spans="2:2">
-      <c r="B24" s="2"/>
+      <c r="B24" s="1"/>
     </row>
     <row r="26" spans="2:2">
-      <c r="B26" s="2"/>
+      <c r="B26" s="1"/>
     </row>
     <row r="28" spans="2:2">
-      <c r="B28" s="2"/>
+      <c r="B28" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>